<commit_message>
Update project files after local changes 10.12.2025
</commit_message>
<xml_diff>
--- a/data/W201.xlsx
+++ b/data/W201.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\py\Git_OrCAD\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{524AE991-66EA-447A-871D-E99471B7114F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{82959428-8E2A-440C-98A9-AA6026C4A462}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="14303" yWindow="-8115" windowWidth="28995" windowHeight="15675" xr2:uid="{8E43C3FC-ABCF-405B-9C0C-A095F821D481}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{8E43C3FC-ABCF-405B-9C0C-A095F821D481}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="43" uniqueCount="39">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="45" uniqueCount="40">
   <si>
     <t>Signal name</t>
   </si>
@@ -142,6 +142,9 @@
   </si>
   <si>
     <t>P2/E</t>
+  </si>
+  <si>
+    <t>TW</t>
   </si>
 </sst>
 </file>
@@ -666,8 +669,14 @@
       <c r="D12" t="s">
         <v>19</v>
       </c>
+      <c r="E12" t="s">
+        <v>39</v>
+      </c>
       <c r="F12">
         <v>20</v>
+      </c>
+      <c r="I12">
+        <v>3</v>
       </c>
       <c r="J12">
         <v>2</v>
@@ -686,6 +695,9 @@
       <c r="D13" t="s">
         <v>19</v>
       </c>
+      <c r="E13" t="s">
+        <v>39</v>
+      </c>
       <c r="F13">
         <v>20</v>
       </c>
@@ -726,6 +738,9 @@
       <c r="F15">
         <v>20</v>
       </c>
+      <c r="I15">
+        <v>3</v>
+      </c>
     </row>
     <row r="16" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
@@ -742,6 +757,9 @@
       </c>
       <c r="F16">
         <v>20</v>
+      </c>
+      <c r="I16">
+        <v>3</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Update project files after local changes 13.12.2025
</commit_message>
<xml_diff>
--- a/data/W201.xlsx
+++ b/data/W201.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\py\Git_OrCAD\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{82959428-8E2A-440C-98A9-AA6026C4A462}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{15B14131-194F-4826-9428-8B6BC8F3DFC8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{8E43C3FC-ABCF-405B-9C0C-A095F821D481}"/>
+    <workbookView xWindow="14303" yWindow="-8115" windowWidth="28995" windowHeight="15675" xr2:uid="{8E43C3FC-ABCF-405B-9C0C-A095F821D481}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="45" uniqueCount="40">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="43" uniqueCount="39">
   <si>
     <t>Signal name</t>
   </si>
@@ -129,22 +129,19 @@
     <t>P1/E</t>
   </si>
   <si>
-    <t>P2/A</t>
-  </si>
-  <si>
-    <t>P2/B</t>
-  </si>
-  <si>
-    <t>P2/C</t>
-  </si>
-  <si>
-    <t>P2/D</t>
-  </si>
-  <si>
-    <t>P2/E</t>
-  </si>
-  <si>
-    <t>TW</t>
+    <t>P2/1</t>
+  </si>
+  <si>
+    <t>P2/2</t>
+  </si>
+  <si>
+    <t>P2/3</t>
+  </si>
+  <si>
+    <t>P2/4</t>
+  </si>
+  <si>
+    <t>P2/5</t>
   </si>
 </sst>
 </file>
@@ -669,17 +666,11 @@
       <c r="D12" t="s">
         <v>19</v>
       </c>
-      <c r="E12" t="s">
-        <v>39</v>
-      </c>
       <c r="F12">
         <v>20</v>
       </c>
       <c r="I12">
-        <v>3</v>
-      </c>
-      <c r="J12">
-        <v>2</v>
+        <v>5</v>
       </c>
     </row>
     <row r="13" spans="1:10" x14ac:dyDescent="0.25">
@@ -695,9 +686,6 @@
       <c r="D13" t="s">
         <v>19</v>
       </c>
-      <c r="E13" t="s">
-        <v>39</v>
-      </c>
       <c r="F13">
         <v>20</v>
       </c>
@@ -718,9 +706,6 @@
       <c r="F14">
         <v>20</v>
       </c>
-      <c r="J14">
-        <v>2</v>
-      </c>
     </row>
     <row r="15" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
@@ -738,9 +723,6 @@
       <c r="F15">
         <v>20</v>
       </c>
-      <c r="I15">
-        <v>3</v>
-      </c>
     </row>
     <row r="16" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
@@ -758,8 +740,8 @@
       <c r="F16">
         <v>20</v>
       </c>
-      <c r="I16">
-        <v>3</v>
+      <c r="J16">
+        <v>1</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Update project files after local changes 14.12.2025
</commit_message>
<xml_diff>
--- a/data/W201.xlsx
+++ b/data/W201.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\py\Git_OrCAD\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{15B14131-194F-4826-9428-8B6BC8F3DFC8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2B1125D0-41B6-434A-9346-217D1E69486F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="14303" yWindow="-8115" windowWidth="28995" windowHeight="15675" xr2:uid="{8E43C3FC-ABCF-405B-9C0C-A095F821D481}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="43" uniqueCount="39">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="45" uniqueCount="40">
   <si>
     <t>Signal name</t>
   </si>
@@ -129,19 +129,22 @@
     <t>P1/E</t>
   </si>
   <si>
-    <t>P2/1</t>
-  </si>
-  <si>
-    <t>P2/2</t>
-  </si>
-  <si>
-    <t>P2/3</t>
-  </si>
-  <si>
-    <t>P2/4</t>
-  </si>
-  <si>
-    <t>P2/5</t>
+    <t>P2/A1</t>
+  </si>
+  <si>
+    <t>P2/A2</t>
+  </si>
+  <si>
+    <t>P2/B3</t>
+  </si>
+  <si>
+    <t>P2/B4</t>
+  </si>
+  <si>
+    <t>TW</t>
+  </si>
+  <si>
+    <t>P2/C5</t>
   </si>
 </sst>
 </file>
@@ -666,6 +669,9 @@
       <c r="D12" t="s">
         <v>19</v>
       </c>
+      <c r="E12" t="s">
+        <v>38</v>
+      </c>
       <c r="F12">
         <v>20</v>
       </c>
@@ -686,6 +692,9 @@
       <c r="D13" t="s">
         <v>19</v>
       </c>
+      <c r="E13" t="s">
+        <v>38</v>
+      </c>
       <c r="F13">
         <v>20</v>
       </c>
@@ -732,7 +741,7 @@
         <v>33</v>
       </c>
       <c r="C16" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="D16" t="s">
         <v>19</v>

</xml_diff>

<commit_message>
Update project files after local changes 21.12.2025
</commit_message>
<xml_diff>
--- a/data/W201.xlsx
+++ b/data/W201.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\py\Git_OrCAD\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2B1125D0-41B6-434A-9346-217D1E69486F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{54B6E1D2-E059-45BA-B22D-B3D45045EBC1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="14303" yWindow="-8115" windowWidth="28995" windowHeight="15675" xr2:uid="{8E43C3FC-ABCF-405B-9C0C-A095F821D481}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{8E43C3FC-ABCF-405B-9C0C-A095F821D481}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -126,9 +126,6 @@
     <t>P1/D</t>
   </si>
   <si>
-    <t>P1/E</t>
-  </si>
-  <si>
     <t>P2/A1</t>
   </si>
   <si>
@@ -145,6 +142,9 @@
   </si>
   <si>
     <t>P2/C5</t>
+  </si>
+  <si>
+    <t>P2/E</t>
   </si>
 </sst>
 </file>
@@ -664,13 +664,13 @@
         <v>29</v>
       </c>
       <c r="C12" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="D12" t="s">
         <v>19</v>
       </c>
       <c r="E12" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="F12">
         <v>20</v>
@@ -687,16 +687,19 @@
         <v>30</v>
       </c>
       <c r="C13" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="D13" t="s">
         <v>19</v>
       </c>
       <c r="E13" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="F13">
         <v>20</v>
+      </c>
+      <c r="I13">
+        <v>3</v>
       </c>
     </row>
     <row r="14" spans="1:10" x14ac:dyDescent="0.25">
@@ -707,13 +710,16 @@
         <v>31</v>
       </c>
       <c r="C14" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="D14" t="s">
         <v>19</v>
       </c>
       <c r="F14">
         <v>20</v>
+      </c>
+      <c r="J14">
+        <v>2</v>
       </c>
     </row>
     <row r="15" spans="1:10" x14ac:dyDescent="0.25">
@@ -724,7 +730,7 @@
         <v>32</v>
       </c>
       <c r="C15" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="D15" t="s">
         <v>19</v>
@@ -738,10 +744,10 @@
         <v>28</v>
       </c>
       <c r="B16" t="s">
-        <v>33</v>
+        <v>39</v>
       </c>
       <c r="C16" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="D16" t="s">
         <v>19</v>

</xml_diff>